<commit_message>
deleted irrelevant ResourcePool code
</commit_message>
<xml_diff>
--- a/Task Point System.xlsx
+++ b/Task Point System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\safaa\Desktop\se116-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B06B8A7B-0E8F-419B-878F-695205A3A40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE51471-B89A-4354-8265-FB54104A20CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
   <si>
     <t>Task ID</t>
   </si>
@@ -129,6 +129,18 @@
   </si>
   <si>
     <t>19.05.2026 16.45</t>
+  </si>
+  <si>
+    <t>BFS search</t>
+  </si>
+  <si>
+    <t>19.05.2026 18.00</t>
+  </si>
+  <si>
+    <t>19.05.2026 21.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tried to understand the BFS search and added the isConnectable / added consumeUtility to Zone class / Made ResourcePool but deleted it after after understanding the logic </t>
   </si>
 </sst>
 </file>
@@ -427,7 +439,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.88671875" customWidth="1"/>
@@ -567,6 +579,29 @@
       </c>
       <c r="G6" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7">
+        <v>60</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Model katmanı guncellendi: Zone kurallari, uretim hesaplamalari ve Service yaricaplari eklendi
</commit_message>
<xml_diff>
--- a/Task Point System.xlsx
+++ b/Task Point System.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\safaa\Desktop\se116-project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayberker/Desktop/se116-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE51471-B89A-4354-8265-FB54104A20CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EDB28EB0-E2D7-2743-9321-77DA23215E3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="23260" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Görev Listesi" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="50">
   <si>
     <t>Task ID</t>
   </si>
@@ -141,13 +141,43 @@
   </si>
   <si>
     <t xml:space="preserve">Tried to understand the BFS search and added the isConnectable / added consumeUtility to Zone class / Made ResourcePool but deleted it after after understanding the logic </t>
+  </si>
+  <si>
+    <t>Ayberk ER</t>
+  </si>
+  <si>
+    <t>Zone class and consumeUtility</t>
+  </si>
+  <si>
+    <t>Housing,Industrial and Commerical classes and level and output calculations</t>
+  </si>
+  <si>
+    <t>The range and service type of services buildings</t>
+  </si>
+  <si>
+    <t>24.05.2026 22.00</t>
+  </si>
+  <si>
+    <t>24.05.2026 23.00</t>
+  </si>
+  <si>
+    <t>23.05.2026 22.00</t>
+  </si>
+  <si>
+    <t>24.05.2026 00.00</t>
+  </si>
+  <si>
+    <t>24.05.2026 17.00</t>
+  </si>
+  <si>
+    <t>24.05.2026 18.00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -159,11 +189,13 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -171,12 +203,14 @@
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -184,6 +218,14 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -208,7 +250,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -216,6 +258,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Köprü" xfId="1" builtinId="8"/>
@@ -232,10 +275,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -439,17 +478,17 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="29.44140625" customWidth="1"/>
-    <col min="6" max="6" width="17.109375" customWidth="1"/>
-    <col min="7" max="7" width="22.21875" customWidth="1"/>
+    <col min="4" max="4" width="72" customWidth="1"/>
+    <col min="6" max="6" width="17.1640625" customWidth="1"/>
+    <col min="7" max="7" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -478,7 +517,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -501,7 +540,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -524,7 +563,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -535,7 +574,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -558,7 +597,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -581,7 +620,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -602,6 +641,66 @@
       </c>
       <c r="G7" t="s">
         <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8">
+        <v>60</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9">
+        <v>50</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10">
+        <v>30</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -619,13 +718,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15.21875" customWidth="1"/>
+    <col min="2" max="2" width="15.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="4" t="s">
         <v>17</v>
       </c>
@@ -642,22 +741,22 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
task point system updated
</commit_message>
<xml_diff>
--- a/Task Point System.xlsx
+++ b/Task Point System.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="78">
   <si>
     <t>Task ID</t>
   </si>
@@ -229,6 +229,15 @@
   </si>
   <si>
     <t>29.05.2026 06.30</t>
+  </si>
+  <si>
+    <t>Implemented the distribution of utilities and resources. And update zones accordingly.</t>
+  </si>
+  <si>
+    <t>30.05.2026 14.00</t>
+  </si>
+  <si>
+    <t>30.05.2026 15.20</t>
   </si>
   <si>
     <t>Developer</t>
@@ -265,7 +274,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="25">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -309,20 +318,6 @@
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -771,150 +766,150 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -923,8 +918,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1186,7 +1179,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultColWidth="12.712962962963" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="7.85185185185185" customWidth="1"/>
@@ -1513,25 +1506,25 @@
       </c>
     </row>
     <row r="15" customHeight="1" spans="1:9">
-      <c r="A15" s="8">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="7" t="s">
         <v>57</v>
       </c>
       <c r="E15">
         <v>70</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="7" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1573,6 +1566,26 @@
       </c>
       <c r="G17" s="7" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="18" customHeight="1" spans="1:7">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18">
+        <v>70</v>
+      </c>
+      <c r="F18" t="s">
+        <v>68</v>
+      </c>
+      <c r="G18" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1599,29 +1612,29 @@
   <sheetData>
     <row r="1" customHeight="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customHeight="1" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" customHeight="1" spans="1:5">
@@ -1631,7 +1644,7 @@
     </row>
     <row r="5" customHeight="1" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented UtilityConsumer interface and integrated it into the base Zone class.
</commit_message>
<xml_diff>
--- a/Task Point System.xlsx
+++ b/Task Point System.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayberker/IdeaProjects/se116-project/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEA54B72-3AF7-054D-A57C-6E51DAB2D343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8580"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Görev Listesi" sheetId="1" r:id="rId1"/>
@@ -28,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="86">
   <si>
     <t>Task ID</t>
   </si>
@@ -262,19 +268,38 @@
   </si>
   <si>
     <t>Ömer Gökberk Gök</t>
+  </si>
+  <si>
+    <t>Bug fixing</t>
+  </si>
+  <si>
+    <t>Fixed UtilityType null pointer in Providers, corrected Euclidean distance formula, fixed ResourcePool consumption logic in distributeResources</t>
+  </si>
+  <si>
+    <t>31.05.2026 00.00</t>
+  </si>
+  <si>
+    <t>30.05.2026 21.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+The commit problems I experienced on Git caused me to spend quite a while, which is why I was only able to push this commit to GitHub a day later.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implemented UtilityConsumer interface and integrated it into the base Zone class. </t>
+  </si>
+  <si>
+    <t>31.05.2026 02.00</t>
+  </si>
+  <si>
+    <t>31.05.2026 03.00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="25">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -320,344 +345,29 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -665,315 +375,38 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="2">
+    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Virgül" xfId="1" builtinId="3"/>
-    <cellStyle name="Para Birimi" xfId="2" builtinId="4"/>
-    <cellStyle name="Yüzde" xfId="3" builtinId="5"/>
-    <cellStyle name="Virgül [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Para Birimi [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Bağlantı" xfId="6" builtinId="8"/>
-    <cellStyle name="Takip Edilen Bağlantı" xfId="7" builtinId="9"/>
-    <cellStyle name="Not" xfId="8" builtinId="10"/>
-    <cellStyle name="Uyarı Metni" xfId="9" builtinId="11"/>
-    <cellStyle name="Başlık" xfId="10" builtinId="15"/>
-    <cellStyle name="Açıklayıcı Metin" xfId="11" builtinId="53"/>
-    <cellStyle name="Başlık 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Başlık 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Başlık 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Başlık 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Giriş" xfId="16" builtinId="20"/>
-    <cellStyle name="Çıktı" xfId="17" builtinId="21"/>
-    <cellStyle name="Hesaplama" xfId="18" builtinId="22"/>
-    <cellStyle name="Hücreyi Kontrol Et" xfId="19" builtinId="23"/>
-    <cellStyle name="Bağlantılı Hücre" xfId="20" builtinId="24"/>
-    <cellStyle name="Toplam" xfId="21" builtinId="25"/>
-    <cellStyle name="İyi" xfId="22" builtinId="26"/>
-    <cellStyle name="Kötü" xfId="23" builtinId="27"/>
-    <cellStyle name="Nötr" xfId="24" builtinId="28"/>
-    <cellStyle name="Vurgu1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Vurgu1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Vurgu1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Vurgu1" xfId="28" builtinId="32"/>
-    <cellStyle name="Vurgu2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Vurgu2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Vurgu2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Vurgu2" xfId="32" builtinId="36"/>
-    <cellStyle name="Vurgu3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Vurgu3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Vurgu3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Vurgu3" xfId="36" builtinId="40"/>
-    <cellStyle name="Vurgu4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Vurgu4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Vurgu4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Vurgu4" xfId="40" builtinId="44"/>
-    <cellStyle name="Vurgu5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Vurgu5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Vurgu5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Vurgu5" xfId="44" builtinId="48"/>
-    <cellStyle name="Vurgu6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Vurgu6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Vurgu6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Vurgu6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1171,25 +604,26 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultColWidth="12.712962962963" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="7.85185185185185" customWidth="1"/>
-    <col min="2" max="2" width="19.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" customWidth="1"/>
     <col min="4" max="4" width="72" customWidth="1"/>
-    <col min="6" max="6" width="17.1388888888889" customWidth="1"/>
-    <col min="7" max="7" width="22.1388888888889" customWidth="1"/>
+    <col min="6" max="6" width="17.1640625" customWidth="1"/>
+    <col min="7" max="7" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.2" spans="1:9">
+    <row r="1" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1218,7 +652,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="13.2" spans="1:9">
+    <row r="2" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1241,7 +675,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="13.2" spans="1:9">
+    <row r="3" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1264,7 +698,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" ht="13.2" spans="1:9">
+    <row r="4" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1284,7 +718,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:9">
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1304,7 +738,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" customHeight="1" spans="1:9">
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1327,7 +761,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="1:9">
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1350,7 +784,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" customHeight="1" spans="1:9">
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1373,202 +807,205 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" customHeight="1" spans="1:9">
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" t="s">
         <v>37</v>
       </c>
       <c r="E9">
         <v>60</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" t="s">
         <v>38</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" customHeight="1" spans="1:9">
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" t="s">
         <v>40</v>
       </c>
       <c r="E10">
         <v>50</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="1:9">
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" t="s">
         <v>36</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" t="s">
         <v>44</v>
       </c>
       <c r="E11">
         <v>30</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="1:9">
+    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" t="s">
         <v>9</v>
       </c>
       <c r="C12" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" t="s">
         <v>47</v>
       </c>
       <c r="E12">
         <v>70</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" t="s">
         <v>48</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="1:9">
+    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" t="s">
         <v>9</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" t="s">
         <v>50</v>
       </c>
       <c r="E13">
         <v>30</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" t="s">
         <v>51</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:9">
+    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" t="s">
         <v>53</v>
       </c>
       <c r="E14">
         <v>40</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" t="s">
         <v>54</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="1:9">
+    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" t="s">
         <v>57</v>
       </c>
       <c r="E15">
         <v>70</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" t="s">
         <v>58</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="16" customHeight="1" spans="1:9">
+      <c r="I15" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" t="s">
         <v>60</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" t="s">
         <v>61</v>
       </c>
       <c r="E16">
         <v>80</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" t="s">
         <v>62</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="17" customHeight="1" spans="1:7">
+    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" t="s">
         <v>64</v>
       </c>
       <c r="E17">
         <v>50</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" t="s">
         <v>65</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="18" customHeight="1" spans="1:7">
+    <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1588,29 +1025,69 @@
         <v>69</v>
       </c>
     </row>
+    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="7">
+        <v>18</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19">
+        <v>70</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="I19" s="8"/>
+    </row>
+    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B20" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20">
+        <v>40</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" display="https://github.com/safeapricot/se116-project/blob/main/README.md"/>
-    <hyperlink ref="H3" r:id="rId2" display="https://github.com/safeapricot/se116-project/blob/main/objectville%202%20mindmap.png"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="H3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="12.712962962963" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="4" outlineLevelCol="4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="17.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="15.1388888888889" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:5">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>70</v>
       </c>
@@ -1627,28 +1104,27 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:5">
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="1:5">
+    <row r="3" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="4" customHeight="1" spans="1:5">
+    <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:5">
+    <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
         <v>77</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
SimulationManager changes, manifest file added.
</commit_message>
<xml_diff>
--- a/Task Point System.xlsx
+++ b/Task Point System.xlsx
@@ -1,40 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayberker/IdeaProjects/se116-project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\safaa\Desktop\se116-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEA54B72-3AF7-054D-A57C-6E51DAB2D343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{266DCAEC-E439-47B2-B9BB-E5E27BEC1FCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Görev Listesi" sheetId="1" r:id="rId1"/>
     <sheet name="Developer List" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="89">
   <si>
     <t>Task ID</t>
   </si>
@@ -293,13 +280,22 @@
   </si>
   <si>
     <t>31.05.2026 03.00</t>
+  </si>
+  <si>
+    <t>Fixed the typos and some methods in SimulationManager, learned the jre file creation</t>
+  </si>
+  <si>
+    <t>01.06.2026 11.00</t>
+  </si>
+  <si>
+    <t>01.06.2026 12.00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -613,17 +609,17 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" customWidth="1"/>
+    <col min="1" max="1" width="7.77734375" customWidth="1"/>
     <col min="2" max="2" width="19.6640625" customWidth="1"/>
     <col min="4" max="4" width="72" customWidth="1"/>
-    <col min="6" max="6" width="17.1640625" customWidth="1"/>
-    <col min="7" max="7" width="22.1640625" customWidth="1"/>
+    <col min="6" max="6" width="17.109375" customWidth="1"/>
+    <col min="7" max="7" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:9" ht="13.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -652,7 +648,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="13" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:9" ht="13.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -675,7 +671,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:9" ht="13.2">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -698,7 +694,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="13" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:9" ht="13.2">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -718,7 +714,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:9" ht="15.75" customHeight="1">
       <c r="A5">
         <v>4</v>
       </c>
@@ -738,7 +734,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:9" ht="15.75" customHeight="1">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -761,7 +757,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:9" ht="15.75" customHeight="1">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -784,7 +780,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:9" ht="15.75" customHeight="1">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -807,7 +803,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:9" ht="15.75" customHeight="1">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -827,7 +823,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:9" ht="15.75" customHeight="1">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -847,7 +843,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:9" ht="15.75" customHeight="1">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -870,7 +866,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:9" ht="15.75" customHeight="1">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -893,7 +889,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:9" ht="15.75" customHeight="1">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -916,7 +912,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:9" ht="15.75" customHeight="1">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -939,7 +935,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:9" ht="15.75" customHeight="1">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -965,7 +961,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:9" ht="15.75" customHeight="1">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -985,7 +981,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:9" ht="15.75" customHeight="1">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1005,7 +1001,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:9" ht="15.75" customHeight="1">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1025,7 +1021,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:9" ht="15.75" customHeight="1">
       <c r="A19" s="7">
         <v>18</v>
       </c>
@@ -1049,7 +1045,10 @@
       </c>
       <c r="I19" s="8"/>
     </row>
-    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
       <c r="B20" s="8" t="s">
         <v>36</v>
       </c>
@@ -1064,6 +1063,34 @@
       </c>
       <c r="G20" s="8" t="s">
         <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>86</v>
+      </c>
+      <c r="E21">
+        <v>30</v>
+      </c>
+      <c r="F21" t="s">
+        <v>87</v>
+      </c>
+      <c r="G21" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1081,13 +1108,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15.1640625" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>70</v>
       </c>
@@ -1104,22 +1131,22 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:5" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:5" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:5" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:5" ht="15.75" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>77</v>
       </c>

</xml_diff>

<commit_message>
Implemented total utility demand calculation and utility absorb.
</commit_message>
<xml_diff>
--- a/Task Point System.xlsx
+++ b/Task Point System.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\safaa\Desktop\se116-project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayberker/IdeaProjects/se116-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE5B3138-903C-44BD-A813-FD2CD537E1EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F62D339D-9D5F-B245-901A-038EC094CA72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="23260" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Görev Listesi" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="98">
   <si>
     <t>Task ID</t>
   </si>
@@ -307,13 +307,22 @@
   </si>
   <si>
     <t>added the manifest file, added the output system to a file that copies console output with System.setOut and made the logs file</t>
+  </si>
+  <si>
+    <t>İmplemented total utility demand calculation and utility absorb via BFS, using polymorphism</t>
+  </si>
+  <si>
+    <t>01.06.2026 23.30</t>
+  </si>
+  <si>
+    <t>01.06.2026 20.00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -646,17 +655,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="7.77734375" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="19.6640625" customWidth="1"/>
     <col min="4" max="4" width="72" customWidth="1"/>
-    <col min="6" max="6" width="17.109375" customWidth="1"/>
-    <col min="7" max="7" width="22.109375" customWidth="1"/>
+    <col min="6" max="6" width="17.1640625" customWidth="1"/>
+    <col min="7" max="7" width="22.1640625" customWidth="1"/>
     <col min="9" max="9" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="13.2">
+    <row r="1" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -685,7 +694,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="13.2">
+    <row r="2" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -708,7 +717,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13.2">
+    <row r="3" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -731,7 +740,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="13.2">
+    <row r="4" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -751,7 +760,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1">
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5">
         <v>4</v>
       </c>
@@ -771,7 +780,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1">
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -794,7 +803,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" customHeight="1">
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -817,7 +826,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" customHeight="1">
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -840,7 +849,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" customHeight="1">
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -860,7 +869,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" customHeight="1">
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -880,7 +889,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75" customHeight="1">
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -903,7 +912,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75" customHeight="1">
+    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -926,7 +935,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.75" customHeight="1">
+    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -949,7 +958,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.75" customHeight="1">
+    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -972,7 +981,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.75" customHeight="1">
+    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -998,7 +1007,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.75" customHeight="1">
+    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1018,7 +1027,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15.75" customHeight="1">
+    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1038,7 +1047,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75" customHeight="1">
+    <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1058,7 +1067,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15.75" customHeight="1">
+    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="7">
         <v>18</v>
       </c>
@@ -1082,7 +1091,7 @@
       </c>
       <c r="I19" s="8"/>
     </row>
-    <row r="20" spans="1:9" ht="15.75" customHeight="1">
+    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1102,7 +1111,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="15.75" customHeight="1">
+    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1125,7 +1134,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.75" customHeight="1">
+    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1154,9 +1163,27 @@
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15.75" customHeight="1">
+    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="11">
         <v>22</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E23">
+        <v>70</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1175,13 +1202,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" customWidth="1"/>
+    <col min="2" max="2" width="15.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" customHeight="1">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>70</v>
       </c>
@@ -1198,22 +1225,22 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" customHeight="1">
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" customHeight="1">
+    <row r="3" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" customHeight="1">
+    <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" customHeight="1">
+    <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
         <v>77</v>
       </c>

</xml_diff>

<commit_message>
Implemented the core game loop in SimulationManager and console output was formatted according to the desired sample output.
</commit_message>
<xml_diff>
--- a/Task Point System.xlsx
+++ b/Task Point System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayberker/IdeaProjects/se116-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F62D339D-9D5F-B245-901A-038EC094CA72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{952FD4F6-C7EE-4A45-A244-9E115B54A3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="23260" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Görev Listesi" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="101">
   <si>
     <t>Task ID</t>
   </si>
@@ -316,6 +316,15 @@
   </si>
   <si>
     <t>01.06.2026 20.00</t>
+  </si>
+  <si>
+    <t>Implemented the core game loop in SimulationManager and console output was formatted according to the desired sample output.</t>
+  </si>
+  <si>
+    <t>03.06.2026 20.30</t>
+  </si>
+  <si>
+    <t>03.06.2026 23.30</t>
   </si>
 </sst>
 </file>
@@ -654,7 +663,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
@@ -1184,6 +1193,26 @@
       </c>
       <c r="G23" s="8" t="s">
         <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="7">
+        <v>23</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E24">
+        <v>70</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Leveling systems have been implemented for all zone classes d applied a consistent, iterative logic structure for level updates.
</commit_message>
<xml_diff>
--- a/Task Point System.xlsx
+++ b/Task Point System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayberker/IdeaProjects/se116-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{952FD4F6-C7EE-4A45-A244-9E115B54A3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{977C63A8-B66C-174A-81D2-814D089A39EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="104">
   <si>
     <t>Task ID</t>
   </si>
@@ -321,10 +321,19 @@
     <t>Implemented the core game loop in SimulationManager and console output was formatted according to the desired sample output.</t>
   </si>
   <si>
-    <t>03.06.2026 20.30</t>
-  </si>
-  <si>
-    <t>03.06.2026 23.30</t>
+    <t>Leveling systems have been implemented for all zone classes d applied a consistent, iterative logic structure for level updates.</t>
+  </si>
+  <si>
+    <t>03.06.2026 19.30</t>
+  </si>
+  <si>
+    <t>03.06.2026 22.00</t>
+  </si>
+  <si>
+    <t>04.06.2026 00.00</t>
+  </si>
+  <si>
+    <t>03.06.2026 22.30</t>
   </si>
 </sst>
 </file>
@@ -663,7 +672,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
@@ -1206,14 +1215,37 @@
         <v>98</v>
       </c>
       <c r="E24">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F24" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="7">
+        <v>24</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G24" s="8" t="s">
-        <v>100</v>
-      </c>
+      <c r="E25">
+        <v>50</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="G26" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Overrode toString methods in Zone classes for better data logging
Refactored Zone subclasses by overriding toString() methods to ensure accurate object state logging instead of memory hash references.
</commit_message>
<xml_diff>
--- a/Task Point System.xlsx
+++ b/Task Point System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fa777143d0771eb9/Belgeler/GitHub/se116-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{D3507CEA-CF63-4E69-B90B-5A7A2460F344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5381818-C751-49E4-93A2-2A69DF188FA9}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{D3507CEA-CF63-4E69-B90B-5A7A2460F344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1FFDA2B-2FFB-411E-8276-B03E27D0E9FA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="111">
   <si>
     <t>Task ID</t>
   </si>
@@ -352,7 +352,22 @@
     <t>Refactored instanceof checks for code consistency, implemented InvalidMapException, and filled missing UtilityConsumer methods in Housing.</t>
   </si>
   <si>
-    <t>04..06.2026 01.00</t>
+    <t>04.06.2026 01.00</t>
+  </si>
+  <si>
+    <t>04.06.2026 02.00</t>
+  </si>
+  <si>
+    <t>03.06.2026  22.00</t>
+  </si>
+  <si>
+    <t>Properly implemented and secured the Commercial class by adding safe map key (containsKey) checks for the Security service to prevent NullPointerException.</t>
+  </si>
+  <si>
+    <t>Fixed map key typos (whitespace issues) and resolved multiple NullPointerException crashes in Housing class by securely integrating hasSecurity, hasHealth, and hasEducation checks.</t>
+  </si>
+  <si>
+    <t>04.06.2026 00.30</t>
   </si>
 </sst>
 </file>
@@ -488,6 +503,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -691,7 +710,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="7.77734375" customWidth="1"/>
@@ -1075,7 +1094,7 @@
         <v>64</v>
       </c>
       <c r="E17">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F17" t="s">
         <v>65</v>
@@ -1304,6 +1323,54 @@
       </c>
       <c r="G27" s="8" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D28" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28">
+        <v>90</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" t="s">
+        <v>109</v>
+      </c>
+      <c r="E29">
+        <v>40</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1363,7 +1430,7 @@
       </c>
       <c r="E2">
         <f>SUM('Görev Listesi'!E:E) / 4</f>
-        <v>347.5</v>
+        <v>382.5</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" customHeight="1">
@@ -1389,15 +1456,15 @@
       </c>
       <c r="B4">
         <f>COUNTIF('Görev Listesi'!B:B, A4)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C4">
         <f>SUMIF('Görev Listesi'!B:B, A4, 'Görev Listesi'!E:E)</f>
-        <v>190</v>
+        <v>330</v>
       </c>
       <c r="D4">
         <f>ROUND((C4 / E2) * 100, 2)</f>
-        <v>54.68</v>
+        <v>86.27</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1">
@@ -1414,7 +1481,7 @@
       </c>
       <c r="D5">
         <f>ROUND((C5 / E2) * 100, 2)</f>
-        <v>51.8</v>
+        <v>47.06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>